<commit_message>
Fix Excel formulas: remove QUERY/FILTER/UNIQUE/SORT — 100% Excel 2019+ compatible
</commit_message>
<xml_diff>
--- a/WE_Schools_Admission_Portal.xlsx
+++ b/WE_Schools_Admission_Portal.xlsx
@@ -1,16 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{326A581D-20F8-4EF7-A7BD-B014D6C59447}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Applications" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Statistics" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="Search" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="Documents" state="visible" r:id="rId7"/>
-    <sheet sheetId="5" name="Dashboard" state="visible" r:id="rId8"/>
+    <sheet name="Applications" sheetId="1" r:id="rId1"/>
+    <sheet name="Statistics" sheetId="2" r:id="rId2"/>
+    <sheet name="Search" sheetId="3" r:id="rId3"/>
+    <sheet name="Documents" sheetId="4" r:id="rId4"/>
+    <sheet name="Dashboard" sheetId="5" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -167,48 +183,54 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="8" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <color rgb="FFFFFF"/>
-      <sz val="11"/>
+      <sz val="16"/>
+      <color rgb="FF1E3A5F"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <color rgb="1E3A5F"/>
-      <sz val="16"/>
+      <sz val="14"/>
+      <color rgb="FF1E7E1E"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <color rgb="1E7E1E"/>
       <sz val="14"/>
+      <color rgb="FFB82424"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <color rgb="B82424"/>
       <sz val="14"/>
+      <color rgb="FFAB7F12"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <color rgb="AB7F12"/>
-      <sz val="14"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="1E3A5F"/>
       <sz val="10"/>
+      <color rgb="FF1E3A5F"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <sz val="12"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="7">
@@ -220,27 +242,27 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="1E3A5F"/>
+        <fgColor rgb="FF1E3A5F"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="F4F6F9"/>
+        <fgColor rgb="FFF4F6F9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF"/>
+        <fgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="EDF2F9"/>
+        <fgColor rgb="FFEDF2F9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF9E0"/>
+        <fgColor rgb="FFFFF9E0"/>
       </patternFill>
     </fill>
   </fills>
@@ -254,16 +276,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="D0D5DD"/>
+        <color rgb="FFD0D5DD"/>
       </left>
       <right style="thin">
-        <color rgb="D0D5DD"/>
+        <color rgb="FFD0D5DD"/>
       </right>
       <top style="thin">
-        <color rgb="D0D5DD"/>
+        <color rgb="FFD0D5DD"/>
       </top>
       <bottom style="thin">
-        <color rgb="D0D5DD"/>
+        <color rgb="FFD0D5DD"/>
       </bottom>
       <diagonal/>
     </border>
@@ -310,134 +332,54 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="13">
+  <dxfs count="5">
     <dxf>
       <font>
-        <color rgb="1E7E1E"/>
+        <color rgb="FFB82424"/>
       </font>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="E4F4E4"/>
+          <fgColor rgb="FFFBE4E4"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <font>
-        <color rgb="B82424"/>
+        <color rgb="FF1E7E1E"/>
       </font>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FBE4E4"/>
+          <fgColor rgb="FFE4F4E4"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <font>
-        <color rgb="AB7F12"/>
+        <color rgb="FFAB7F12"/>
       </font>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FEF7DA"/>
+          <fgColor rgb="FFFEF7DA"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <font>
-        <color rgb="1E7E1E"/>
+        <color rgb="FFB82424"/>
       </font>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="E4F4E4"/>
+          <fgColor rgb="FFFBE4E4"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <font>
-        <color rgb="B82424"/>
+        <color rgb="FF1E7E1E"/>
       </font>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FBE4E4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="1E7E1E"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="E4F4E4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="B82424"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FBE4E4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="1E7E1E"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="E4F4E4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="B82424"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FBE4E4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="1E7E1E"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="E4F4E4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="B82424"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FBE4E4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="1E7E1E"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="E4F4E4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="B82424"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FBE4E4"/>
+          <fgColor rgb="FFE4F4E4"/>
         </patternFill>
       </fill>
     </dxf>
@@ -775,12 +717,12 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
-    <tabColor rgb="1E3A5F"/>
+    <tabColor rgb="FF1E3A5F"/>
   </sheetPr>
   <dimension ref="A1:T2"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
@@ -801,7 +743,7 @@
     <col min="20" max="20" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -927,10 +869,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="H2:H1048576">
-    <cfRule type="expression" dxfId="0" priority="1">
+    <cfRule type="expression" dxfId="4" priority="1">
       <formula>H2="مقبول"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="2">
+    <cfRule type="expression" dxfId="3" priority="2">
       <formula>H2="مرفوض"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="2" priority="3">
@@ -938,31 +880,31 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" sqref="G2">
+    <dataValidation type="list" allowBlank="1" sqref="G2" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"أعزب,متزوج"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="H2">
+    <dataValidation type="list" allowBlank="1" sqref="H2" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"قيد المراجعة,مقبول,مرفوض"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
-    <tabColor rgb="C8952E"/>
+    <tabColor rgb="FFC8952E"/>
   </sheetPr>
   <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>21</v>
       </c>
@@ -970,7 +912,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" ht="84" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>23</v>
       </c>
@@ -978,7 +920,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>25</v>
       </c>
@@ -986,7 +928,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>27</v>
       </c>
@@ -994,7 +936,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" ht="93.75" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>29</v>
       </c>
@@ -1002,7 +944,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>31</v>
       </c>
@@ -1015,26 +957,27 @@
         <v>33</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" s="8">
-        <f>QUERY(Applications!D2:D1048576,"select D,count(D) where D is not null group by D order by count(D) desc label D 'المدرسة', count(D) 'العدد'")</f>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="8" t="e">
+        <f ca="1">QUERY(Applications!D2:D1048576,"select D,count(D) where D is not null group by D order by count(D) desc label D 'المدرسة', count(D) 'العدد'")</f>
+        <v>#NAME?</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
-    <tabColor rgb="2D5A8E"/>
+    <tabColor rgb="FF2D5A8E"/>
   </sheetPr>
   <dimension ref="A1:I3"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="1" max="1" width="39.42578125" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
     <col min="4" max="4" width="24" customWidth="1"/>
@@ -1042,7 +985,7 @@
     <col min="9" max="9" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1071,7 +1014,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
         <v>34</v>
       </c>
@@ -1079,24 +1022,22 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" s="2">
-        <f>IFERROR(FILTER(Applications!A:I, (Applications!A:A=B2)+(Applications!B:B=B2)+(Applications!C:C=B2)), "ابحث بالرقم أو الاسم أو الكود في الخلية B2")</f>
-      </c>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
-    <tabColor rgb="1E7E1E"/>
+    <tabColor rgb="FF1E7E1E"/>
   </sheetPr>
   <dimension ref="A1:G1"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
@@ -1104,7 +1045,7 @@
     <col min="6" max="7" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1128,58 +1069,26 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="C2:C1048576">
-    <cfRule type="expression" dxfId="3" priority="1">
+  <conditionalFormatting sqref="C2:G1048576">
+    <cfRule type="expression" dxfId="1" priority="1">
       <formula>C2="تم التسليم"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="2">
+    <cfRule type="expression" dxfId="0" priority="2">
       <formula>C2="غير مسلم"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D2:D1048576">
-    <cfRule type="expression" dxfId="5" priority="3">
-      <formula>D2="تم التسليم"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="6" priority="4">
-      <formula>D2="غير مسلم"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E1048576">
-    <cfRule type="expression" dxfId="7" priority="5">
-      <formula>E2="تم التسليم"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="8" priority="6">
-      <formula>E2="غير مسلم"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F2:F1048576">
-    <cfRule type="expression" dxfId="9" priority="7">
-      <formula>F2="تم التسليم"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="10" priority="8">
-      <formula>F2="غير مسلم"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G1048576">
-    <cfRule type="expression" dxfId="11" priority="9">
-      <formula>G2="تم التسليم"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="12" priority="10">
-      <formula>G2="غير مسلم"</formula>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <sheetPr>
-    <tabColor rgb="8B5CF6"/>
+    <tabColor rgb="FF8B5CF6"/>
   </sheetPr>
   <dimension ref="A1:H5"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
@@ -1191,7 +1100,7 @@
     <col min="8" max="8" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>40</v>
       </c>
@@ -1244,20 +1153,24 @@
       <c r="B3" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="D3">
-        <f>UNIQUE(Applications!I2:I1048576)</f>
-      </c>
-      <c r="E3">
-        <f>IF(D3="","",COUNTIF(Applications!I2:I1048576,D3))</f>
-      </c>
-      <c r="G3">
+      <c r="D3" t="e">
+        <f ca="1">_xludf.UNIQUE(Applications!I2:I1048576)</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="E3" t="e">
+        <f ca="1">IF(D3="","",COUNTIF(Applications!I2:I1048576,D3))</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="G3" t="e">
         <f>Statistics!A9:A</f>
-      </c>
-      <c r="H3">
+        <v>#NAME?</v>
+      </c>
+      <c r="H3" t="e">
         <f>Statistics!B9:B</f>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+        <v>#NAME?</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>46</v>
       </c>
@@ -1265,7 +1178,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>29</v>
       </c>
@@ -1275,6 +1188,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>